<commit_message>
refactor: tampilkan tiap komponen nilai terpisah per kolom di samping (tidak dirata-rata)
</commit_message>
<xml_diff>
--- a/nilai-nilai/pola-2026/POLA_PAIK6808_2025_2_A.xlsx
+++ b/nilai-nilai/pola-2026/POLA_PAIK6808_2025_2_A.xlsx
@@ -16,7 +16,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="3">
     <font>
       <name val="Calibri"/>
       <strike val="0"/>
@@ -28,6 +28,9 @@
       <strike val="0"/>
       <color rgb="FFFFFFFF"/>
       <sz val="11"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -47,7 +50,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
@@ -63,6 +66,10 @@
     </xf>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -431,22 +438,28 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M55"/>
+  <dimension ref="A1:T55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4" outlineLevelRow="0"/>
   <cols>
-    <col width="17.567139" bestFit="1" customWidth="1" min="1" max="1"/>
-    <col width="47.131348" bestFit="1" customWidth="1" min="2" max="2"/>
-    <col width="10.568848" bestFit="1" customWidth="1" min="3" max="3"/>
-    <col width="8.140869" bestFit="1" customWidth="1" min="4" max="4"/>
-    <col width="57.700195" bestFit="1" customWidth="1" min="5" max="5"/>
-    <col width="45.845947" bestFit="1" customWidth="1" min="6" max="6"/>
-    <col width="36.419678" bestFit="1" customWidth="1" min="7" max="7"/>
-    <col width="35.2771" bestFit="1" customWidth="1" min="8" max="8"/>
-    <col width="35.2771" bestFit="1" customWidth="1" min="9" max="9"/>
-    <col width="31.706543" bestFit="1" customWidth="1" min="10" max="10"/>
-    <col width="37.705078" bestFit="1" customWidth="1" min="11" max="11"/>
-    <col width="35.2771" bestFit="1" customWidth="1" min="12" max="12"/>
-    <col width="21.137695" bestFit="1" customWidth="1" min="13" max="13"/>
+    <col width="17.567139" bestFit="1" customWidth="1" style="5" min="1" max="1"/>
+    <col width="47.131348" bestFit="1" customWidth="1" style="5" min="2" max="2"/>
+    <col width="10.568848" bestFit="1" customWidth="1" style="5" min="3" max="3"/>
+    <col width="8.140869" bestFit="1" customWidth="1" style="5" min="4" max="4"/>
+    <col width="57.700195" bestFit="1" customWidth="1" style="5" min="5" max="5"/>
+    <col width="45.845947" bestFit="1" customWidth="1" style="5" min="6" max="6"/>
+    <col width="36.419678" bestFit="1" customWidth="1" style="5" min="7" max="7"/>
+    <col width="35.2771" bestFit="1" customWidth="1" style="5" min="8" max="8"/>
+    <col width="35.2771" bestFit="1" customWidth="1" style="5" min="9" max="9"/>
+    <col width="31.706543" bestFit="1" customWidth="1" style="5" min="10" max="10"/>
+    <col width="37.705078" bestFit="1" customWidth="1" style="5" min="11" max="11"/>
+    <col width="35.2771" bestFit="1" customWidth="1" style="5" min="12" max="12"/>
+    <col width="21.137695" bestFit="1" customWidth="1" style="5" min="13" max="13"/>
+    <col width="16" customWidth="1" style="5" min="15" max="15"/>
+    <col width="16" customWidth="1" style="5" min="16" max="16"/>
+    <col width="16" customWidth="1" style="5" min="17" max="17"/>
+    <col width="16" customWidth="1" style="5" min="18" max="18"/>
+    <col width="16" customWidth="1" style="5" min="19" max="19"/>
+    <col width="16" customWidth="1" style="5" min="20" max="20"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -580,6 +593,41 @@
           <t>Nilai Bobot (0-4)</t>
         </is>
       </c>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t>|</t>
+        </is>
+      </c>
+      <c r="O7" s="6" t="inlineStr">
+        <is>
+          <t>Classification Task (Intermediate)</t>
+        </is>
+      </c>
+      <c r="P7" s="6" t="inlineStr">
+        <is>
+          <t>Evaluation Metric Quiz</t>
+        </is>
+      </c>
+      <c r="Q7" s="6" t="inlineStr">
+        <is>
+          <t>Manual Classification Task (Beginner)</t>
+        </is>
+      </c>
+      <c r="R7" s="6" t="inlineStr">
+        <is>
+          <t>Oral</t>
+        </is>
+      </c>
+      <c r="S7" s="6" t="inlineStr">
+        <is>
+          <t>Arsitektur</t>
+        </is>
+      </c>
+      <c r="T7" s="6" t="inlineStr">
+        <is>
+          <t>Proyek (Presentasi + Keaktifan)</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="0" t="inlineStr">
@@ -601,13 +649,9 @@
         </is>
       </c>
       <c r="E8" s="3" t="n"/>
-      <c r="F8" s="3" t="n">
-        <v>84.33</v>
-      </c>
+      <c r="F8" s="3" t="n"/>
       <c r="G8" s="3" t="n"/>
-      <c r="H8" s="3" t="n">
-        <v>94.43000000000001</v>
-      </c>
+      <c r="H8" s="3" t="n"/>
       <c r="I8" s="3" t="n"/>
       <c r="J8" s="3" t="n"/>
       <c r="K8" s="4">
@@ -622,6 +666,29 @@
         <f>IF(AND(K8&gt;=80, K8&lt;=100), "4", IF(AND(K8&gt;=70, K8&lt;=79.99999999999), "3", IF(AND(K8&gt;=60, K8&lt;=69.9999999999), "2", IF(AND(K8&gt;=51, K8&lt;=59.999999999), "1", IF(AND(K8&gt;=0, K8&lt;=50.999999999), "0",  "0"  )  )  )  )  ) </f>
         <v/>
       </c>
+      <c r="N8" t="inlineStr">
+        <is>
+          <t>|</t>
+        </is>
+      </c>
+      <c r="O8" t="n">
+        <v>10</v>
+      </c>
+      <c r="P8" t="n">
+        <v>10</v>
+      </c>
+      <c r="Q8" t="n">
+        <v>8.33</v>
+      </c>
+      <c r="R8" t="n">
+        <v>8</v>
+      </c>
+      <c r="S8" t="n">
+        <v>9.300000000000001</v>
+      </c>
+      <c r="T8" t="n">
+        <v>80</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="0" t="inlineStr">
@@ -643,13 +710,9 @@
         </is>
       </c>
       <c r="E9" s="3" t="n"/>
-      <c r="F9" s="3" t="n">
-        <v>85</v>
-      </c>
+      <c r="F9" s="3" t="n"/>
       <c r="G9" s="3" t="n"/>
-      <c r="H9" s="3" t="n">
-        <v>74.43000000000001</v>
-      </c>
+      <c r="H9" s="3" t="n"/>
       <c r="I9" s="3" t="n"/>
       <c r="J9" s="3" t="n"/>
       <c r="K9" s="4">
@@ -664,6 +727,29 @@
         <f>IF(AND(K9&gt;=80, K9&lt;=100), "4", IF(AND(K9&gt;=70, K9&lt;=79.99999999999), "3", IF(AND(K9&gt;=60, K9&lt;=69.9999999999), "2", IF(AND(K9&gt;=51, K9&lt;=59.999999999), "1", IF(AND(K9&gt;=0, K9&lt;=50.999999999), "0",  "0"  )  )  )  )  ) </f>
         <v/>
       </c>
+      <c r="N9" t="inlineStr">
+        <is>
+          <t>|</t>
+        </is>
+      </c>
+      <c r="O9" t="n">
+        <v>9</v>
+      </c>
+      <c r="P9" t="n">
+        <v>10</v>
+      </c>
+      <c r="Q9" t="n">
+        <v>3.33</v>
+      </c>
+      <c r="R9" t="n">
+        <v>8.699999999999999</v>
+      </c>
+      <c r="S9" t="n">
+        <v>8.800000000000001</v>
+      </c>
+      <c r="T9" t="n">
+        <v>80</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="0" t="inlineStr">
@@ -685,13 +771,9 @@
         </is>
       </c>
       <c r="E10" s="3" t="n"/>
-      <c r="F10" s="3" t="n">
-        <v>92.67</v>
-      </c>
+      <c r="F10" s="3" t="n"/>
       <c r="G10" s="3" t="n"/>
-      <c r="H10" s="3" t="n">
-        <v>82.23</v>
-      </c>
+      <c r="H10" s="3" t="n"/>
       <c r="I10" s="3" t="n"/>
       <c r="J10" s="3" t="n"/>
       <c r="K10" s="4">
@@ -706,6 +788,29 @@
         <f>IF(AND(K10&gt;=80, K10&lt;=100), "4", IF(AND(K10&gt;=70, K10&lt;=79.99999999999), "3", IF(AND(K10&gt;=60, K10&lt;=69.9999999999), "2", IF(AND(K10&gt;=51, K10&lt;=59.999999999), "1", IF(AND(K10&gt;=0, K10&lt;=50.999999999), "0",  "0"  )  )  )  )  ) </f>
         <v/>
       </c>
+      <c r="N10" t="inlineStr">
+        <is>
+          <t>|</t>
+        </is>
+      </c>
+      <c r="O10" t="n">
+        <v>9.67</v>
+      </c>
+      <c r="P10" t="n">
+        <v>5</v>
+      </c>
+      <c r="Q10" t="n">
+        <v>10</v>
+      </c>
+      <c r="R10" t="n">
+        <v>9.300000000000001</v>
+      </c>
+      <c r="S10" t="n">
+        <v>9</v>
+      </c>
+      <c r="T10" t="n">
+        <v>95</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="0" t="inlineStr">
@@ -727,13 +832,9 @@
         </is>
       </c>
       <c r="E11" s="3" t="n"/>
-      <c r="F11" s="3" t="n">
-        <v>27.33</v>
-      </c>
+      <c r="F11" s="3" t="n"/>
       <c r="G11" s="3" t="n"/>
-      <c r="H11" s="3" t="n">
-        <v>0</v>
-      </c>
+      <c r="H11" s="3" t="n"/>
       <c r="I11" s="3" t="n"/>
       <c r="J11" s="4" t="n"/>
       <c r="K11" s="4">
@@ -748,6 +849,14 @@
         <f>IF(AND(K11&gt;=80, K11&lt;=100), "4", IF(AND(K11&gt;=70, K11&lt;=79.99999999999), "3", IF(AND(K11&gt;=60, K11&lt;=69.9999999999), "2", IF(AND(K11&gt;=51, K11&lt;=59.999999999), "1", IF(AND(K11&gt;=0, K11&lt;=50.999999999), "0",  "0"  )  )  )  )  ) </f>
         <v/>
       </c>
+      <c r="N11" t="inlineStr">
+        <is>
+          <t>|</t>
+        </is>
+      </c>
+      <c r="T11" t="n">
+        <v>82</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="0" t="inlineStr">
@@ -769,13 +878,9 @@
         </is>
       </c>
       <c r="E12" s="3" t="n"/>
-      <c r="F12" s="3" t="n">
-        <v>80.67</v>
-      </c>
+      <c r="F12" s="3" t="n"/>
       <c r="G12" s="3" t="n"/>
-      <c r="H12" s="3" t="n">
-        <v>77.77</v>
-      </c>
+      <c r="H12" s="3" t="n"/>
       <c r="I12" s="3" t="n"/>
       <c r="J12" s="3" t="n"/>
       <c r="K12" s="4">
@@ -790,6 +895,29 @@
         <f>IF(AND(K12&gt;=80, K12&lt;=100), "4", IF(AND(K12&gt;=70, K12&lt;=79.99999999999), "3", IF(AND(K12&gt;=60, K12&lt;=69.9999999999), "2", IF(AND(K12&gt;=51, K12&lt;=59.999999999), "1", IF(AND(K12&gt;=0, K12&lt;=50.999999999), "0",  "0"  )  )  )  )  ) </f>
         <v/>
       </c>
+      <c r="N12" t="inlineStr">
+        <is>
+          <t>|</t>
+        </is>
+      </c>
+      <c r="O12" t="n">
+        <v>10</v>
+      </c>
+      <c r="P12" t="n">
+        <v>10</v>
+      </c>
+      <c r="Q12" t="n">
+        <v>3.33</v>
+      </c>
+      <c r="R12" t="n">
+        <v>7.5</v>
+      </c>
+      <c r="S12" t="n">
+        <v>8.699999999999999</v>
+      </c>
+      <c r="T12" t="n">
+        <v>80</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="0" t="inlineStr">
@@ -811,13 +939,9 @@
         </is>
       </c>
       <c r="E13" s="3" t="n"/>
-      <c r="F13" s="3" t="n">
-        <v>86.33</v>
-      </c>
+      <c r="F13" s="3" t="n"/>
       <c r="G13" s="3" t="n"/>
-      <c r="H13" s="3" t="n">
-        <v>37.77</v>
-      </c>
+      <c r="H13" s="3" t="n"/>
       <c r="I13" s="3" t="n"/>
       <c r="J13" s="3" t="n"/>
       <c r="K13" s="4">
@@ -832,6 +956,29 @@
         <f>IF(AND(K13&gt;=80, K13&lt;=100), "4", IF(AND(K13&gt;=70, K13&lt;=79.99999999999), "3", IF(AND(K13&gt;=60, K13&lt;=69.9999999999), "2", IF(AND(K13&gt;=51, K13&lt;=59.999999999), "1", IF(AND(K13&gt;=0, K13&lt;=50.999999999), "0",  "0"  )  )  )  )  ) </f>
         <v/>
       </c>
+      <c r="N13" t="inlineStr">
+        <is>
+          <t>|</t>
+        </is>
+      </c>
+      <c r="O13" t="n">
+        <v>8</v>
+      </c>
+      <c r="P13" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q13" t="n">
+        <v>3.33</v>
+      </c>
+      <c r="R13" t="n">
+        <v>9.199999999999999</v>
+      </c>
+      <c r="S13" t="n">
+        <v>8.699999999999999</v>
+      </c>
+      <c r="T13" t="n">
+        <v>80</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="0" t="inlineStr">
@@ -853,13 +1000,9 @@
         </is>
       </c>
       <c r="E14" s="3" t="n"/>
-      <c r="F14" s="3" t="n">
-        <v>82</v>
-      </c>
+      <c r="F14" s="3" t="n"/>
       <c r="G14" s="3" t="n"/>
-      <c r="H14" s="3" t="n">
-        <v>91.67</v>
-      </c>
+      <c r="H14" s="3" t="n"/>
       <c r="I14" s="3" t="n"/>
       <c r="J14" s="3" t="n"/>
       <c r="K14" s="4">
@@ -874,6 +1017,29 @@
         <f>IF(AND(K14&gt;=80, K14&lt;=100), "4", IF(AND(K14&gt;=70, K14&lt;=79.99999999999), "3", IF(AND(K14&gt;=60, K14&lt;=69.9999999999), "2", IF(AND(K14&gt;=51, K14&lt;=59.999999999), "1", IF(AND(K14&gt;=0, K14&lt;=50.999999999), "0",  "0"  )  )  )  )  ) </f>
         <v/>
       </c>
+      <c r="N14" t="inlineStr">
+        <is>
+          <t>|</t>
+        </is>
+      </c>
+      <c r="O14" t="n">
+        <v>10</v>
+      </c>
+      <c r="P14" t="n">
+        <v>7.5</v>
+      </c>
+      <c r="Q14" t="n">
+        <v>10</v>
+      </c>
+      <c r="R14" t="n">
+        <v>6</v>
+      </c>
+      <c r="S14" t="n">
+        <v>9.4</v>
+      </c>
+      <c r="T14" t="n">
+        <v>92</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="0" t="inlineStr">
@@ -895,13 +1061,9 @@
         </is>
       </c>
       <c r="E15" s="3" t="n"/>
-      <c r="F15" s="3" t="n">
-        <v>84</v>
-      </c>
+      <c r="F15" s="3" t="n"/>
       <c r="G15" s="3" t="n"/>
-      <c r="H15" s="3" t="n">
-        <v>72.2</v>
-      </c>
+      <c r="H15" s="3" t="n"/>
       <c r="I15" s="3" t="n"/>
       <c r="J15" s="3" t="n"/>
       <c r="K15" s="4">
@@ -916,6 +1078,29 @@
         <f>IF(AND(K15&gt;=80, K15&lt;=100), "4", IF(AND(K15&gt;=70, K15&lt;=79.99999999999), "3", IF(AND(K15&gt;=60, K15&lt;=69.9999999999), "2", IF(AND(K15&gt;=51, K15&lt;=59.999999999), "1", IF(AND(K15&gt;=0, K15&lt;=50.999999999), "0",  "0"  )  )  )  )  ) </f>
         <v/>
       </c>
+      <c r="N15" t="inlineStr">
+        <is>
+          <t>|</t>
+        </is>
+      </c>
+      <c r="O15" t="n">
+        <v>8.33</v>
+      </c>
+      <c r="P15" t="n">
+        <v>10</v>
+      </c>
+      <c r="Q15" t="n">
+        <v>3.33</v>
+      </c>
+      <c r="R15" t="n">
+        <v>8.5</v>
+      </c>
+      <c r="S15" t="n">
+        <v>8.699999999999999</v>
+      </c>
+      <c r="T15" t="n">
+        <v>80</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="0" t="inlineStr">
@@ -937,13 +1122,9 @@
         </is>
       </c>
       <c r="E16" s="3" t="n"/>
-      <c r="F16" s="3" t="n">
-        <v>60.67</v>
-      </c>
+      <c r="F16" s="3" t="n"/>
       <c r="G16" s="3" t="n"/>
-      <c r="H16" s="3" t="n">
-        <v>69.47</v>
-      </c>
+      <c r="H16" s="3" t="n"/>
       <c r="I16" s="3" t="n"/>
       <c r="J16" s="3" t="n"/>
       <c r="K16" s="4">
@@ -958,6 +1139,29 @@
         <f>IF(AND(K16&gt;=80, K16&lt;=100), "4", IF(AND(K16&gt;=70, K16&lt;=79.99999999999), "3", IF(AND(K16&gt;=60, K16&lt;=69.9999999999), "2", IF(AND(K16&gt;=51, K16&lt;=59.999999999), "1", IF(AND(K16&gt;=0, K16&lt;=50.999999999), "0",  "0"  )  )  )  )  ) </f>
         <v/>
       </c>
+      <c r="N16" t="inlineStr">
+        <is>
+          <t>|</t>
+        </is>
+      </c>
+      <c r="O16" t="n">
+        <v>6.67</v>
+      </c>
+      <c r="P16" t="n">
+        <v>7.5</v>
+      </c>
+      <c r="Q16" t="n">
+        <v>6.67</v>
+      </c>
+      <c r="R16" t="n">
+        <v>9.4</v>
+      </c>
+      <c r="S16" t="n">
+        <v>8.800000000000001</v>
+      </c>
+      <c r="T16" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="0" t="inlineStr">
@@ -979,13 +1183,9 @@
         </is>
       </c>
       <c r="E17" s="3" t="n"/>
-      <c r="F17" s="3" t="n">
-        <v>55.33</v>
-      </c>
+      <c r="F17" s="3" t="n"/>
       <c r="G17" s="3" t="n"/>
-      <c r="H17" s="3" t="n">
-        <v>48.9</v>
-      </c>
+      <c r="H17" s="3" t="n"/>
       <c r="I17" s="3" t="n"/>
       <c r="J17" s="4" t="n"/>
       <c r="K17" s="4">
@@ -1000,6 +1200,23 @@
         <f>IF(AND(K17&gt;=80, K17&lt;=100), "4", IF(AND(K17&gt;=70, K17&lt;=79.99999999999), "3", IF(AND(K17&gt;=60, K17&lt;=69.9999999999), "2", IF(AND(K17&gt;=51, K17&lt;=59.999999999), "1", IF(AND(K17&gt;=0, K17&lt;=50.999999999), "0",  "0"  )  )  )  )  ) </f>
         <v/>
       </c>
+      <c r="N17" t="inlineStr">
+        <is>
+          <t>|</t>
+        </is>
+      </c>
+      <c r="O17" t="n">
+        <v>8</v>
+      </c>
+      <c r="Q17" t="n">
+        <v>6.67</v>
+      </c>
+      <c r="S17" t="n">
+        <v>8.6</v>
+      </c>
+      <c r="T17" t="n">
+        <v>80</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="0" t="inlineStr">
@@ -1021,13 +1238,9 @@
         </is>
       </c>
       <c r="E18" s="3" t="n"/>
-      <c r="F18" s="3" t="n">
-        <v>29</v>
-      </c>
+      <c r="F18" s="3" t="n"/>
       <c r="G18" s="3" t="n"/>
-      <c r="H18" s="3" t="n">
-        <v>0</v>
-      </c>
+      <c r="H18" s="3" t="n"/>
       <c r="I18" s="3" t="n"/>
       <c r="J18" s="4" t="n"/>
       <c r="K18" s="4">
@@ -1042,6 +1255,14 @@
         <f>IF(AND(K18&gt;=80, K18&lt;=100), "4", IF(AND(K18&gt;=70, K18&lt;=79.99999999999), "3", IF(AND(K18&gt;=60, K18&lt;=69.9999999999), "2", IF(AND(K18&gt;=51, K18&lt;=59.999999999), "1", IF(AND(K18&gt;=0, K18&lt;=50.999999999), "0",  "0"  )  )  )  )  ) </f>
         <v/>
       </c>
+      <c r="N18" t="inlineStr">
+        <is>
+          <t>|</t>
+        </is>
+      </c>
+      <c r="T18" t="n">
+        <v>87</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="0" t="inlineStr">
@@ -1063,13 +1284,9 @@
         </is>
       </c>
       <c r="E19" s="3" t="n"/>
-      <c r="F19" s="3" t="n">
-        <v>90.67</v>
-      </c>
+      <c r="F19" s="3" t="n"/>
       <c r="G19" s="3" t="n"/>
-      <c r="H19" s="3" t="n">
-        <v>92.2</v>
-      </c>
+      <c r="H19" s="3" t="n"/>
       <c r="I19" s="3" t="n"/>
       <c r="J19" s="3" t="n"/>
       <c r="K19" s="4">
@@ -1084,6 +1301,29 @@
         <f>IF(AND(K19&gt;=80, K19&lt;=100), "4", IF(AND(K19&gt;=70, K19&lt;=79.99999999999), "3", IF(AND(K19&gt;=60, K19&lt;=69.9999999999), "2", IF(AND(K19&gt;=51, K19&lt;=59.999999999), "1", IF(AND(K19&gt;=0, K19&lt;=50.999999999), "0",  "0"  )  )  )  )  ) </f>
         <v/>
       </c>
+      <c r="N19" t="inlineStr">
+        <is>
+          <t>|</t>
+        </is>
+      </c>
+      <c r="O19" t="n">
+        <v>9.33</v>
+      </c>
+      <c r="P19" t="n">
+        <v>10</v>
+      </c>
+      <c r="Q19" t="n">
+        <v>8.33</v>
+      </c>
+      <c r="R19" t="n">
+        <v>9.300000000000001</v>
+      </c>
+      <c r="S19" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="T19" t="n">
+        <v>90</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="0" t="inlineStr">
@@ -1105,13 +1345,9 @@
         </is>
       </c>
       <c r="E20" s="3" t="n"/>
-      <c r="F20" s="3" t="n">
-        <v>27.33</v>
-      </c>
+      <c r="F20" s="3" t="n"/>
       <c r="G20" s="3" t="n"/>
-      <c r="H20" s="3" t="n">
-        <v>0</v>
-      </c>
+      <c r="H20" s="3" t="n"/>
       <c r="I20" s="3" t="n"/>
       <c r="J20" s="4" t="n"/>
       <c r="K20" s="4">
@@ -1126,6 +1362,14 @@
         <f>IF(AND(K20&gt;=80, K20&lt;=100), "4", IF(AND(K20&gt;=70, K20&lt;=79.99999999999), "3", IF(AND(K20&gt;=60, K20&lt;=69.9999999999), "2", IF(AND(K20&gt;=51, K20&lt;=59.999999999), "1", IF(AND(K20&gt;=0, K20&lt;=50.999999999), "0",  "0"  )  )  )  )  ) </f>
         <v/>
       </c>
+      <c r="N20" t="inlineStr">
+        <is>
+          <t>|</t>
+        </is>
+      </c>
+      <c r="T20" t="n">
+        <v>82</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="0" t="inlineStr">
@@ -1147,13 +1391,9 @@
         </is>
       </c>
       <c r="E21" s="3" t="n"/>
-      <c r="F21" s="3" t="n">
-        <v>87.33</v>
-      </c>
+      <c r="F21" s="3" t="n"/>
       <c r="G21" s="3" t="n"/>
-      <c r="H21" s="3" t="n">
-        <v>47.8</v>
-      </c>
+      <c r="H21" s="3" t="n"/>
       <c r="I21" s="3" t="n"/>
       <c r="J21" s="3" t="n"/>
       <c r="K21" s="4">
@@ -1168,6 +1408,29 @@
         <f>IF(AND(K21&gt;=80, K21&lt;=100), "4", IF(AND(K21&gt;=70, K21&lt;=79.99999999999), "3", IF(AND(K21&gt;=60, K21&lt;=69.9999999999), "2", IF(AND(K21&gt;=51, K21&lt;=59.999999999), "1", IF(AND(K21&gt;=0, K21&lt;=50.999999999), "0",  "0"  )  )  )  )  ) </f>
         <v/>
       </c>
+      <c r="N21" t="inlineStr">
+        <is>
+          <t>|</t>
+        </is>
+      </c>
+      <c r="O21" t="n">
+        <v>7.67</v>
+      </c>
+      <c r="P21" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q21" t="n">
+        <v>6.67</v>
+      </c>
+      <c r="R21" t="n">
+        <v>8.300000000000001</v>
+      </c>
+      <c r="S21" t="n">
+        <v>9.199999999999999</v>
+      </c>
+      <c r="T21" t="n">
+        <v>87</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="0" t="inlineStr">
@@ -1189,13 +1452,9 @@
         </is>
       </c>
       <c r="E22" s="3" t="n"/>
-      <c r="F22" s="3" t="n">
-        <v>89</v>
-      </c>
+      <c r="F22" s="3" t="n"/>
       <c r="G22" s="3" t="n"/>
-      <c r="H22" s="3" t="n">
-        <v>90.56999999999999</v>
-      </c>
+      <c r="H22" s="3" t="n"/>
       <c r="I22" s="3" t="n"/>
       <c r="J22" s="3" t="n"/>
       <c r="K22" s="4">
@@ -1210,6 +1469,29 @@
         <f>IF(AND(K22&gt;=80, K22&lt;=100), "4", IF(AND(K22&gt;=70, K22&lt;=79.99999999999), "3", IF(AND(K22&gt;=60, K22&lt;=69.9999999999), "2", IF(AND(K22&gt;=51, K22&lt;=59.999999999), "1", IF(AND(K22&gt;=0, K22&lt;=50.999999999), "0",  "0"  )  )  )  )  ) </f>
         <v/>
       </c>
+      <c r="N22" t="inlineStr">
+        <is>
+          <t>|</t>
+        </is>
+      </c>
+      <c r="O22" t="n">
+        <v>9.67</v>
+      </c>
+      <c r="P22" t="n">
+        <v>7.5</v>
+      </c>
+      <c r="Q22" t="n">
+        <v>10</v>
+      </c>
+      <c r="R22" t="n">
+        <v>9</v>
+      </c>
+      <c r="S22" t="n">
+        <v>9</v>
+      </c>
+      <c r="T22" t="n">
+        <v>87</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="0" t="inlineStr">
@@ -1231,13 +1513,9 @@
         </is>
       </c>
       <c r="E23" s="3" t="n"/>
-      <c r="F23" s="3" t="n">
-        <v>28.33</v>
-      </c>
+      <c r="F23" s="3" t="n"/>
       <c r="G23" s="3" t="n"/>
-      <c r="H23" s="3" t="n">
-        <v>0</v>
-      </c>
+      <c r="H23" s="3" t="n"/>
       <c r="I23" s="3" t="n"/>
       <c r="J23" s="4" t="n"/>
       <c r="K23" s="4">
@@ -1252,6 +1530,14 @@
         <f>IF(AND(K23&gt;=80, K23&lt;=100), "4", IF(AND(K23&gt;=70, K23&lt;=79.99999999999), "3", IF(AND(K23&gt;=60, K23&lt;=69.9999999999), "2", IF(AND(K23&gt;=51, K23&lt;=59.999999999), "1", IF(AND(K23&gt;=0, K23&lt;=50.999999999), "0",  "0"  )  )  )  )  ) </f>
         <v/>
       </c>
+      <c r="N23" t="inlineStr">
+        <is>
+          <t>|</t>
+        </is>
+      </c>
+      <c r="T23" t="n">
+        <v>85</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="0" t="inlineStr">
@@ -1273,13 +1559,9 @@
         </is>
       </c>
       <c r="E24" s="3" t="n"/>
-      <c r="F24" s="3" t="n">
-        <v>57</v>
-      </c>
+      <c r="F24" s="3" t="n"/>
       <c r="G24" s="3" t="n"/>
-      <c r="H24" s="3" t="n">
-        <v>86.67</v>
-      </c>
+      <c r="H24" s="3" t="n"/>
       <c r="I24" s="3" t="n"/>
       <c r="J24" s="3" t="n"/>
       <c r="K24" s="4">
@@ -1294,6 +1576,29 @@
         <f>IF(AND(K24&gt;=80, K24&lt;=100), "4", IF(AND(K24&gt;=70, K24&lt;=79.99999999999), "3", IF(AND(K24&gt;=60, K24&lt;=69.9999999999), "2", IF(AND(K24&gt;=51, K24&lt;=59.999999999), "1", IF(AND(K24&gt;=0, K24&lt;=50.999999999), "0",  "0"  )  )  )  )  ) </f>
         <v/>
       </c>
+      <c r="N24" t="inlineStr">
+        <is>
+          <t>|</t>
+        </is>
+      </c>
+      <c r="O24" t="n">
+        <v>9.33</v>
+      </c>
+      <c r="P24" t="n">
+        <v>10</v>
+      </c>
+      <c r="Q24" t="n">
+        <v>6.67</v>
+      </c>
+      <c r="R24" t="n">
+        <v>9.199999999999999</v>
+      </c>
+      <c r="S24" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="T24" t="n">
+        <v>-10</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="0" t="inlineStr">
@@ -1315,13 +1620,9 @@
         </is>
       </c>
       <c r="E25" s="3" t="n"/>
-      <c r="F25" s="3" t="n">
-        <v>81</v>
-      </c>
+      <c r="F25" s="3" t="n"/>
       <c r="G25" s="3" t="n"/>
-      <c r="H25" s="3" t="n">
-        <v>82.77</v>
-      </c>
+      <c r="H25" s="3" t="n"/>
       <c r="I25" s="3" t="n"/>
       <c r="J25" s="3" t="n"/>
       <c r="K25" s="4">
@@ -1336,6 +1637,29 @@
         <f>IF(AND(K25&gt;=80, K25&lt;=100), "4", IF(AND(K25&gt;=70, K25&lt;=79.99999999999), "3", IF(AND(K25&gt;=60, K25&lt;=69.9999999999), "2", IF(AND(K25&gt;=51, K25&lt;=59.999999999), "1", IF(AND(K25&gt;=0, K25&lt;=50.999999999), "0",  "0"  )  )  )  )  ) </f>
         <v/>
       </c>
+      <c r="N25" t="inlineStr">
+        <is>
+          <t>|</t>
+        </is>
+      </c>
+      <c r="O25" t="n">
+        <v>9</v>
+      </c>
+      <c r="P25" t="n">
+        <v>7.5</v>
+      </c>
+      <c r="Q25" t="n">
+        <v>8.33</v>
+      </c>
+      <c r="R25" t="n">
+        <v>7.8</v>
+      </c>
+      <c r="S25" t="n">
+        <v>8.300000000000001</v>
+      </c>
+      <c r="T25" t="n">
+        <v>82</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="0" t="inlineStr">
@@ -1357,13 +1681,9 @@
         </is>
       </c>
       <c r="E26" s="3" t="n"/>
-      <c r="F26" s="3" t="n">
-        <v>86</v>
-      </c>
+      <c r="F26" s="3" t="n"/>
       <c r="G26" s="3" t="n"/>
-      <c r="H26" s="3" t="n">
-        <v>51.13</v>
-      </c>
+      <c r="H26" s="3" t="n"/>
       <c r="I26" s="3" t="n"/>
       <c r="J26" s="3" t="n"/>
       <c r="K26" s="4">
@@ -1378,6 +1698,29 @@
         <f>IF(AND(K26&gt;=80, K26&lt;=100), "4", IF(AND(K26&gt;=70, K26&lt;=79.99999999999), "3", IF(AND(K26&gt;=60, K26&lt;=69.9999999999), "2", IF(AND(K26&gt;=51, K26&lt;=59.999999999), "1", IF(AND(K26&gt;=0, K26&lt;=50.999999999), "0",  "0"  )  )  )  )  ) </f>
         <v/>
       </c>
+      <c r="N26" t="inlineStr">
+        <is>
+          <t>|</t>
+        </is>
+      </c>
+      <c r="O26" t="n">
+        <v>8.67</v>
+      </c>
+      <c r="P26" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q26" t="n">
+        <v>6.67</v>
+      </c>
+      <c r="R26" t="n">
+        <v>8.5</v>
+      </c>
+      <c r="S26" t="n">
+        <v>8.6</v>
+      </c>
+      <c r="T26" t="n">
+        <v>87</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="0" t="inlineStr">
@@ -1399,13 +1742,9 @@
         </is>
       </c>
       <c r="E27" s="3" t="n"/>
-      <c r="F27" s="3" t="n">
-        <v>82.33</v>
-      </c>
+      <c r="F27" s="3" t="n"/>
       <c r="G27" s="3" t="n"/>
-      <c r="H27" s="3" t="n">
-        <v>72.77</v>
-      </c>
+      <c r="H27" s="3" t="n"/>
       <c r="I27" s="3" t="n"/>
       <c r="J27" s="3" t="n"/>
       <c r="K27" s="4">
@@ -1420,6 +1759,29 @@
         <f>IF(AND(K27&gt;=80, K27&lt;=100), "4", IF(AND(K27&gt;=70, K27&lt;=79.99999999999), "3", IF(AND(K27&gt;=60, K27&lt;=69.9999999999), "2", IF(AND(K27&gt;=51, K27&lt;=59.999999999), "1", IF(AND(K27&gt;=0, K27&lt;=50.999999999), "0",  "0"  )  )  )  )  ) </f>
         <v/>
       </c>
+      <c r="N27" t="inlineStr">
+        <is>
+          <t>|</t>
+        </is>
+      </c>
+      <c r="O27" t="n">
+        <v>6</v>
+      </c>
+      <c r="P27" t="n">
+        <v>7.5</v>
+      </c>
+      <c r="Q27" t="n">
+        <v>8.33</v>
+      </c>
+      <c r="R27" t="n">
+        <v>8.199999999999999</v>
+      </c>
+      <c r="S27" t="n">
+        <v>8.5</v>
+      </c>
+      <c r="T27" t="n">
+        <v>80</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="0" t="inlineStr">
@@ -1441,13 +1803,9 @@
         </is>
       </c>
       <c r="E28" s="3" t="n"/>
-      <c r="F28" s="3" t="n">
-        <v>58</v>
-      </c>
+      <c r="F28" s="3" t="n"/>
       <c r="G28" s="3" t="n"/>
-      <c r="H28" s="3" t="n">
-        <v>57.77</v>
-      </c>
+      <c r="H28" s="3" t="n"/>
       <c r="I28" s="3" t="n"/>
       <c r="J28" s="3" t="n"/>
       <c r="K28" s="4">
@@ -1462,6 +1820,26 @@
         <f>IF(AND(K28&gt;=80, K28&lt;=100), "4", IF(AND(K28&gt;=70, K28&lt;=79.99999999999), "3", IF(AND(K28&gt;=60, K28&lt;=69.9999999999), "2", IF(AND(K28&gt;=51, K28&lt;=59.999999999), "1", IF(AND(K28&gt;=0, K28&lt;=50.999999999), "0",  "0"  )  )  )  )  ) </f>
         <v/>
       </c>
+      <c r="N28" t="inlineStr">
+        <is>
+          <t>|</t>
+        </is>
+      </c>
+      <c r="O28" t="n">
+        <v>9</v>
+      </c>
+      <c r="Q28" t="n">
+        <v>8.33</v>
+      </c>
+      <c r="R28" t="n">
+        <v>8.5</v>
+      </c>
+      <c r="S28" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="T28" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="0" t="inlineStr">
@@ -1483,13 +1861,9 @@
         </is>
       </c>
       <c r="E29" s="3" t="n"/>
-      <c r="F29" s="3" t="n">
-        <v>86</v>
-      </c>
+      <c r="F29" s="3" t="n"/>
       <c r="G29" s="3" t="n"/>
-      <c r="H29" s="3" t="n">
-        <v>94.43000000000001</v>
-      </c>
+      <c r="H29" s="3" t="n"/>
       <c r="I29" s="3" t="n"/>
       <c r="J29" s="3" t="n"/>
       <c r="K29" s="4">
@@ -1504,6 +1878,29 @@
         <f>IF(AND(K29&gt;=80, K29&lt;=100), "4", IF(AND(K29&gt;=70, K29&lt;=79.99999999999), "3", IF(AND(K29&gt;=60, K29&lt;=69.9999999999), "2", IF(AND(K29&gt;=51, K29&lt;=59.999999999), "1", IF(AND(K29&gt;=0, K29&lt;=50.999999999), "0",  "0"  )  )  )  )  ) </f>
         <v/>
       </c>
+      <c r="N29" t="inlineStr">
+        <is>
+          <t>|</t>
+        </is>
+      </c>
+      <c r="O29" t="n">
+        <v>10</v>
+      </c>
+      <c r="P29" t="n">
+        <v>10</v>
+      </c>
+      <c r="Q29" t="n">
+        <v>8.33</v>
+      </c>
+      <c r="R29" t="n">
+        <v>8.300000000000001</v>
+      </c>
+      <c r="S29" t="n">
+        <v>9.5</v>
+      </c>
+      <c r="T29" t="n">
+        <v>80</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="0" t="inlineStr">
@@ -1525,13 +1922,9 @@
         </is>
       </c>
       <c r="E30" s="3" t="n"/>
-      <c r="F30" s="3" t="n">
-        <v>26.67</v>
-      </c>
+      <c r="F30" s="3" t="n"/>
       <c r="G30" s="3" t="n"/>
-      <c r="H30" s="3" t="n">
-        <v>75.56999999999999</v>
-      </c>
+      <c r="H30" s="3" t="n"/>
       <c r="I30" s="3" t="n"/>
       <c r="J30" s="4" t="n"/>
       <c r="K30" s="4">
@@ -1546,6 +1939,23 @@
         <f>IF(AND(K30&gt;=80, K30&lt;=100), "4", IF(AND(K30&gt;=70, K30&lt;=79.99999999999), "3", IF(AND(K30&gt;=60, K30&lt;=69.9999999999), "2", IF(AND(K30&gt;=51, K30&lt;=59.999999999), "1", IF(AND(K30&gt;=0, K30&lt;=50.999999999), "0",  "0"  )  )  )  )  ) </f>
         <v/>
       </c>
+      <c r="N30" t="inlineStr">
+        <is>
+          <t>|</t>
+        </is>
+      </c>
+      <c r="O30" t="n">
+        <v>7.67</v>
+      </c>
+      <c r="P30" t="n">
+        <v>10</v>
+      </c>
+      <c r="Q30" t="n">
+        <v>5</v>
+      </c>
+      <c r="T30" t="n">
+        <v>80</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="0" t="inlineStr">
@@ -1567,13 +1977,9 @@
         </is>
       </c>
       <c r="E31" s="3" t="n"/>
-      <c r="F31" s="3" t="n">
-        <v>85</v>
-      </c>
+      <c r="F31" s="3" t="n"/>
       <c r="G31" s="3" t="n"/>
-      <c r="H31" s="3" t="n">
-        <v>80</v>
-      </c>
+      <c r="H31" s="3" t="n"/>
       <c r="I31" s="3" t="n"/>
       <c r="J31" s="3" t="n"/>
       <c r="K31" s="4">
@@ -1588,6 +1994,29 @@
         <f>IF(AND(K31&gt;=80, K31&lt;=100), "4", IF(AND(K31&gt;=70, K31&lt;=79.99999999999), "3", IF(AND(K31&gt;=60, K31&lt;=69.9999999999), "2", IF(AND(K31&gt;=51, K31&lt;=59.999999999), "1", IF(AND(K31&gt;=0, K31&lt;=50.999999999), "0",  "0"  )  )  )  )  ) </f>
         <v/>
       </c>
+      <c r="N31" t="inlineStr">
+        <is>
+          <t>|</t>
+        </is>
+      </c>
+      <c r="O31" t="n">
+        <v>9</v>
+      </c>
+      <c r="P31" t="n">
+        <v>10</v>
+      </c>
+      <c r="Q31" t="n">
+        <v>5</v>
+      </c>
+      <c r="R31" t="n">
+        <v>8.5</v>
+      </c>
+      <c r="S31" t="n">
+        <v>9</v>
+      </c>
+      <c r="T31" t="n">
+        <v>80</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="0" t="inlineStr">
@@ -1609,13 +2038,9 @@
         </is>
       </c>
       <c r="E32" s="3" t="n"/>
-      <c r="F32" s="3" t="n">
-        <v>52.33</v>
-      </c>
+      <c r="F32" s="3" t="n"/>
       <c r="G32" s="3" t="n"/>
-      <c r="H32" s="3" t="n">
-        <v>0</v>
-      </c>
+      <c r="H32" s="3" t="n"/>
       <c r="I32" s="3" t="n"/>
       <c r="J32" s="3" t="n"/>
       <c r="K32" s="4">
@@ -1630,6 +2055,23 @@
         <f>IF(AND(K32&gt;=80, K32&lt;=100), "4", IF(AND(K32&gt;=70, K32&lt;=79.99999999999), "3", IF(AND(K32&gt;=60, K32&lt;=69.9999999999), "2", IF(AND(K32&gt;=51, K32&lt;=59.999999999), "1", IF(AND(K32&gt;=0, K32&lt;=50.999999999), "0",  "0"  )  )  )  )  ) </f>
         <v/>
       </c>
+      <c r="N32" t="inlineStr">
+        <is>
+          <t>|</t>
+        </is>
+      </c>
+      <c r="P32" t="n">
+        <v>0</v>
+      </c>
+      <c r="R32" t="n">
+        <v>7.3</v>
+      </c>
+      <c r="S32" t="n">
+        <v>9.4</v>
+      </c>
+      <c r="T32" t="n">
+        <v>-10</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="0" t="inlineStr">
@@ -1651,13 +2093,9 @@
         </is>
       </c>
       <c r="E33" s="3" t="n"/>
-      <c r="F33" s="3" t="n">
-        <v>29.33</v>
-      </c>
+      <c r="F33" s="3" t="n"/>
       <c r="G33" s="3" t="n"/>
-      <c r="H33" s="3" t="n">
-        <v>0</v>
-      </c>
+      <c r="H33" s="3" t="n"/>
       <c r="I33" s="3" t="n"/>
       <c r="J33" s="4" t="n"/>
       <c r="K33" s="4">
@@ -1672,6 +2110,17 @@
         <f>IF(AND(K33&gt;=80, K33&lt;=100), "4", IF(AND(K33&gt;=70, K33&lt;=79.99999999999), "3", IF(AND(K33&gt;=60, K33&lt;=69.9999999999), "2", IF(AND(K33&gt;=51, K33&lt;=59.999999999), "1", IF(AND(K33&gt;=0, K33&lt;=50.999999999), "0",  "0"  )  )  )  )  ) </f>
         <v/>
       </c>
+      <c r="N33" t="inlineStr">
+        <is>
+          <t>|</t>
+        </is>
+      </c>
+      <c r="S33" t="n">
+        <v>8.800000000000001</v>
+      </c>
+      <c r="T33" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="0" t="inlineStr">
@@ -1693,13 +2142,9 @@
         </is>
       </c>
       <c r="E34" s="3" t="n"/>
-      <c r="F34" s="3" t="n">
-        <v>57.67</v>
-      </c>
+      <c r="F34" s="3" t="n"/>
       <c r="G34" s="3" t="n"/>
-      <c r="H34" s="3" t="n">
-        <v>54.43</v>
-      </c>
+      <c r="H34" s="3" t="n"/>
       <c r="I34" s="3" t="n"/>
       <c r="J34" s="3" t="n"/>
       <c r="K34" s="4">
@@ -1714,6 +2159,26 @@
         <f>IF(AND(K34&gt;=80, K34&lt;=100), "4", IF(AND(K34&gt;=70, K34&lt;=79.99999999999), "3", IF(AND(K34&gt;=60, K34&lt;=69.9999999999), "2", IF(AND(K34&gt;=51, K34&lt;=59.999999999), "1", IF(AND(K34&gt;=0, K34&lt;=50.999999999), "0",  "0"  )  )  )  )  ) </f>
         <v/>
       </c>
+      <c r="N34" t="inlineStr">
+        <is>
+          <t>|</t>
+        </is>
+      </c>
+      <c r="O34" t="n">
+        <v>8</v>
+      </c>
+      <c r="Q34" t="n">
+        <v>8.33</v>
+      </c>
+      <c r="R34" t="n">
+        <v>8.5</v>
+      </c>
+      <c r="S34" t="n">
+        <v>8.800000000000001</v>
+      </c>
+      <c r="T34" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="0" t="inlineStr">
@@ -1735,13 +2200,9 @@
         </is>
       </c>
       <c r="E35" s="3" t="n"/>
-      <c r="F35" s="3" t="n">
-        <v>81</v>
-      </c>
+      <c r="F35" s="3" t="n"/>
       <c r="G35" s="3" t="n"/>
-      <c r="H35" s="3" t="n">
-        <v>25</v>
-      </c>
+      <c r="H35" s="3" t="n"/>
       <c r="I35" s="3" t="n"/>
       <c r="J35" s="3" t="n"/>
       <c r="K35" s="4">
@@ -1756,6 +2217,23 @@
         <f>IF(AND(K35&gt;=80, K35&lt;=100), "4", IF(AND(K35&gt;=70, K35&lt;=79.99999999999), "3", IF(AND(K35&gt;=60, K35&lt;=69.9999999999), "2", IF(AND(K35&gt;=51, K35&lt;=59.999999999), "1", IF(AND(K35&gt;=0, K35&lt;=50.999999999), "0",  "0"  )  )  )  )  ) </f>
         <v/>
       </c>
+      <c r="N35" t="inlineStr">
+        <is>
+          <t>|</t>
+        </is>
+      </c>
+      <c r="P35" t="n">
+        <v>7.5</v>
+      </c>
+      <c r="R35" t="n">
+        <v>8</v>
+      </c>
+      <c r="S35" t="n">
+        <v>8.6</v>
+      </c>
+      <c r="T35" t="n">
+        <v>77</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="0" t="inlineStr">
@@ -1777,13 +2255,9 @@
         </is>
       </c>
       <c r="E36" s="3" t="n"/>
-      <c r="F36" s="3" t="n">
-        <v>53.33</v>
-      </c>
+      <c r="F36" s="3" t="n"/>
       <c r="G36" s="3" t="n"/>
-      <c r="H36" s="3" t="n">
-        <v>34.43</v>
-      </c>
+      <c r="H36" s="3" t="n"/>
       <c r="I36" s="3" t="n"/>
       <c r="J36" s="3" t="n"/>
       <c r="K36" s="4">
@@ -1798,6 +2272,26 @@
         <f>IF(AND(K36&gt;=80, K36&lt;=100), "4", IF(AND(K36&gt;=70, K36&lt;=79.99999999999), "3", IF(AND(K36&gt;=60, K36&lt;=69.9999999999), "2", IF(AND(K36&gt;=51, K36&lt;=59.999999999), "1", IF(AND(K36&gt;=0, K36&lt;=50.999999999), "0",  "0"  )  )  )  )  ) </f>
         <v/>
       </c>
+      <c r="N36" t="inlineStr">
+        <is>
+          <t>|</t>
+        </is>
+      </c>
+      <c r="O36" t="n">
+        <v>7</v>
+      </c>
+      <c r="Q36" t="n">
+        <v>3.33</v>
+      </c>
+      <c r="R36" t="n">
+        <v>7</v>
+      </c>
+      <c r="S36" t="n">
+        <v>9</v>
+      </c>
+      <c r="T36" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="0" t="inlineStr">
@@ -1819,13 +2313,9 @@
         </is>
       </c>
       <c r="E37" s="3" t="n"/>
-      <c r="F37" s="3" t="n">
-        <v>83</v>
-      </c>
+      <c r="F37" s="3" t="n"/>
       <c r="G37" s="3" t="n"/>
-      <c r="H37" s="3" t="n">
-        <v>90.56999999999999</v>
-      </c>
+      <c r="H37" s="3" t="n"/>
       <c r="I37" s="3" t="n"/>
       <c r="J37" s="3" t="n"/>
       <c r="K37" s="4">
@@ -1840,6 +2330,29 @@
         <f>IF(AND(K37&gt;=80, K37&lt;=100), "4", IF(AND(K37&gt;=70, K37&lt;=79.99999999999), "3", IF(AND(K37&gt;=60, K37&lt;=69.9999999999), "2", IF(AND(K37&gt;=51, K37&lt;=59.999999999), "1", IF(AND(K37&gt;=0, K37&lt;=50.999999999), "0",  "0"  )  )  )  )  ) </f>
         <v/>
       </c>
+      <c r="N37" t="inlineStr">
+        <is>
+          <t>|</t>
+        </is>
+      </c>
+      <c r="O37" t="n">
+        <v>9.67</v>
+      </c>
+      <c r="P37" t="n">
+        <v>7.5</v>
+      </c>
+      <c r="Q37" t="n">
+        <v>10</v>
+      </c>
+      <c r="R37" t="n">
+        <v>8</v>
+      </c>
+      <c r="S37" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="T37" t="n">
+        <v>80</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="0" t="inlineStr">
@@ -1861,13 +2374,9 @@
         </is>
       </c>
       <c r="E38" s="3" t="n"/>
-      <c r="F38" s="3" t="n">
-        <v>85.67</v>
-      </c>
+      <c r="F38" s="3" t="n"/>
       <c r="G38" s="3" t="n"/>
-      <c r="H38" s="3" t="n">
-        <v>56.67</v>
-      </c>
+      <c r="H38" s="3" t="n"/>
       <c r="I38" s="3" t="n"/>
       <c r="J38" s="3" t="n"/>
       <c r="K38" s="4">
@@ -1882,6 +2391,29 @@
         <f>IF(AND(K38&gt;=80, K38&lt;=100), "4", IF(AND(K38&gt;=70, K38&lt;=79.99999999999), "3", IF(AND(K38&gt;=60, K38&lt;=69.9999999999), "2", IF(AND(K38&gt;=51, K38&lt;=59.999999999), "1", IF(AND(K38&gt;=0, K38&lt;=50.999999999), "0",  "0"  )  )  )  )  ) </f>
         <v/>
       </c>
+      <c r="N38" t="inlineStr">
+        <is>
+          <t>|</t>
+        </is>
+      </c>
+      <c r="O38" t="n">
+        <v>8.67</v>
+      </c>
+      <c r="P38" t="n">
+        <v>5</v>
+      </c>
+      <c r="Q38" t="n">
+        <v>3.33</v>
+      </c>
+      <c r="R38" t="n">
+        <v>8.300000000000001</v>
+      </c>
+      <c r="S38" t="n">
+        <v>8.699999999999999</v>
+      </c>
+      <c r="T38" t="n">
+        <v>87</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="0" t="inlineStr">
@@ -1903,13 +2435,9 @@
         </is>
       </c>
       <c r="E39" s="3" t="n"/>
-      <c r="F39" s="3" t="n">
-        <v>55.67</v>
-      </c>
+      <c r="F39" s="3" t="n"/>
       <c r="G39" s="3" t="n"/>
-      <c r="H39" s="3" t="n">
-        <v>97.77</v>
-      </c>
+      <c r="H39" s="3" t="n"/>
       <c r="I39" s="3" t="n"/>
       <c r="J39" s="3" t="n"/>
       <c r="K39" s="4">
@@ -1924,6 +2452,29 @@
         <f>IF(AND(K39&gt;=80, K39&lt;=100), "4", IF(AND(K39&gt;=70, K39&lt;=79.99999999999), "3", IF(AND(K39&gt;=60, K39&lt;=69.9999999999), "2", IF(AND(K39&gt;=51, K39&lt;=59.999999999), "1", IF(AND(K39&gt;=0, K39&lt;=50.999999999), "0",  "0"  )  )  )  )  ) </f>
         <v/>
       </c>
+      <c r="N39" t="inlineStr">
+        <is>
+          <t>|</t>
+        </is>
+      </c>
+      <c r="O39" t="n">
+        <v>9.33</v>
+      </c>
+      <c r="P39" t="n">
+        <v>10</v>
+      </c>
+      <c r="Q39" t="n">
+        <v>10</v>
+      </c>
+      <c r="R39" t="n">
+        <v>7.5</v>
+      </c>
+      <c r="S39" t="n">
+        <v>9.199999999999999</v>
+      </c>
+      <c r="T39" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="0" t="inlineStr">
@@ -1945,13 +2496,9 @@
         </is>
       </c>
       <c r="E40" s="3" t="n"/>
-      <c r="F40" s="3" t="n">
-        <v>-3.33</v>
-      </c>
+      <c r="F40" s="3" t="n"/>
       <c r="G40" s="3" t="n"/>
-      <c r="H40" s="3" t="n">
-        <v>0</v>
-      </c>
+      <c r="H40" s="3" t="n"/>
       <c r="I40" s="3" t="n"/>
       <c r="J40" s="4" t="n"/>
       <c r="K40" s="4">
@@ -1966,6 +2513,14 @@
         <f>IF(AND(K40&gt;=80, K40&lt;=100), "4", IF(AND(K40&gt;=70, K40&lt;=79.99999999999), "3", IF(AND(K40&gt;=60, K40&lt;=69.9999999999), "2", IF(AND(K40&gt;=51, K40&lt;=59.999999999), "1", IF(AND(K40&gt;=0, K40&lt;=50.999999999), "0",  "0"  )  )  )  )  ) </f>
         <v/>
       </c>
+      <c r="N40" t="inlineStr">
+        <is>
+          <t>|</t>
+        </is>
+      </c>
+      <c r="T40" t="n">
+        <v>-10</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="0" t="inlineStr">
@@ -1987,13 +2542,9 @@
         </is>
       </c>
       <c r="E41" s="3" t="n"/>
-      <c r="F41" s="3" t="n">
-        <v>56.33</v>
-      </c>
+      <c r="F41" s="3" t="n"/>
       <c r="G41" s="3" t="n"/>
-      <c r="H41" s="3" t="n">
-        <v>93.33</v>
-      </c>
+      <c r="H41" s="3" t="n"/>
       <c r="I41" s="3" t="n"/>
       <c r="J41" s="3" t="n"/>
       <c r="K41" s="4">
@@ -2008,6 +2559,29 @@
         <f>IF(AND(K41&gt;=80, K41&lt;=100), "4", IF(AND(K41&gt;=70, K41&lt;=79.99999999999), "3", IF(AND(K41&gt;=60, K41&lt;=69.9999999999), "2", IF(AND(K41&gt;=51, K41&lt;=59.999999999), "1", IF(AND(K41&gt;=0, K41&lt;=50.999999999), "0",  "0"  )  )  )  )  ) </f>
         <v/>
       </c>
+      <c r="N41" t="inlineStr">
+        <is>
+          <t>|</t>
+        </is>
+      </c>
+      <c r="O41" t="n">
+        <v>9.67</v>
+      </c>
+      <c r="P41" t="n">
+        <v>10</v>
+      </c>
+      <c r="Q41" t="n">
+        <v>8.33</v>
+      </c>
+      <c r="R41" t="n">
+        <v>8</v>
+      </c>
+      <c r="S41" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="T41" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="0" t="inlineStr">
@@ -2029,13 +2603,9 @@
         </is>
       </c>
       <c r="E42" s="3" t="n"/>
-      <c r="F42" s="3" t="n">
-        <v>61.67</v>
-      </c>
+      <c r="F42" s="3" t="n"/>
       <c r="G42" s="3" t="n"/>
-      <c r="H42" s="3" t="n">
-        <v>100</v>
-      </c>
+      <c r="H42" s="3" t="n"/>
       <c r="I42" s="3" t="n"/>
       <c r="J42" s="3" t="n"/>
       <c r="K42" s="4">
@@ -2050,6 +2620,29 @@
         <f>IF(AND(K42&gt;=80, K42&lt;=100), "4", IF(AND(K42&gt;=70, K42&lt;=79.99999999999), "3", IF(AND(K42&gt;=60, K42&lt;=69.9999999999), "2", IF(AND(K42&gt;=51, K42&lt;=59.999999999), "1", IF(AND(K42&gt;=0, K42&lt;=50.999999999), "0",  "0"  )  )  )  )  ) </f>
         <v/>
       </c>
+      <c r="N42" t="inlineStr">
+        <is>
+          <t>|</t>
+        </is>
+      </c>
+      <c r="O42" t="n">
+        <v>10</v>
+      </c>
+      <c r="P42" t="n">
+        <v>10</v>
+      </c>
+      <c r="Q42" t="n">
+        <v>10</v>
+      </c>
+      <c r="R42" t="n">
+        <v>9</v>
+      </c>
+      <c r="S42" t="n">
+        <v>9.5</v>
+      </c>
+      <c r="T42" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="0" t="inlineStr">
@@ -2071,13 +2664,9 @@
         </is>
       </c>
       <c r="E43" s="3" t="n"/>
-      <c r="F43" s="3" t="n">
-        <v>50.33</v>
-      </c>
+      <c r="F43" s="3" t="n"/>
       <c r="G43" s="3" t="n"/>
-      <c r="H43" s="3" t="n">
-        <v>81.09999999999999</v>
-      </c>
+      <c r="H43" s="3" t="n"/>
       <c r="I43" s="3" t="n"/>
       <c r="J43" s="3" t="n"/>
       <c r="K43" s="4">
@@ -2092,6 +2681,29 @@
         <f>IF(AND(K43&gt;=80, K43&lt;=100), "4", IF(AND(K43&gt;=70, K43&lt;=79.99999999999), "3", IF(AND(K43&gt;=60, K43&lt;=69.9999999999), "2", IF(AND(K43&gt;=51, K43&lt;=59.999999999), "1", IF(AND(K43&gt;=0, K43&lt;=50.999999999), "0",  "0"  )  )  )  )  ) </f>
         <v/>
       </c>
+      <c r="N43" t="inlineStr">
+        <is>
+          <t>|</t>
+        </is>
+      </c>
+      <c r="O43" t="n">
+        <v>9.33</v>
+      </c>
+      <c r="P43" t="n">
+        <v>5</v>
+      </c>
+      <c r="Q43" t="n">
+        <v>10</v>
+      </c>
+      <c r="R43" t="n">
+        <v>7.3</v>
+      </c>
+      <c r="S43" t="n">
+        <v>7.8</v>
+      </c>
+      <c r="T43" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="0" t="inlineStr">
@@ -2113,13 +2725,9 @@
         </is>
       </c>
       <c r="E44" s="3" t="n"/>
-      <c r="F44" s="3" t="n">
-        <v>90</v>
-      </c>
+      <c r="F44" s="3" t="n"/>
       <c r="G44" s="3" t="n"/>
-      <c r="H44" s="3" t="n">
-        <v>93.33</v>
-      </c>
+      <c r="H44" s="3" t="n"/>
       <c r="I44" s="3" t="n"/>
       <c r="J44" s="3" t="n"/>
       <c r="K44" s="4">
@@ -2134,6 +2742,29 @@
         <f>IF(AND(K44&gt;=80, K44&lt;=100), "4", IF(AND(K44&gt;=70, K44&lt;=79.99999999999), "3", IF(AND(K44&gt;=60, K44&lt;=69.9999999999), "2", IF(AND(K44&gt;=51, K44&lt;=59.999999999), "1", IF(AND(K44&gt;=0, K44&lt;=50.999999999), "0",  "0"  )  )  )  )  ) </f>
         <v/>
       </c>
+      <c r="N44" t="inlineStr">
+        <is>
+          <t>|</t>
+        </is>
+      </c>
+      <c r="O44" t="n">
+        <v>9.67</v>
+      </c>
+      <c r="P44" t="n">
+        <v>10</v>
+      </c>
+      <c r="Q44" t="n">
+        <v>8.33</v>
+      </c>
+      <c r="R44" t="n">
+        <v>9</v>
+      </c>
+      <c r="S44" t="n">
+        <v>9</v>
+      </c>
+      <c r="T44" t="n">
+        <v>90</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="0" t="inlineStr">
@@ -2155,13 +2786,9 @@
         </is>
       </c>
       <c r="E45" s="3" t="n"/>
-      <c r="F45" s="3" t="n">
-        <v>78</v>
-      </c>
+      <c r="F45" s="3" t="n"/>
       <c r="G45" s="3" t="n"/>
-      <c r="H45" s="3" t="n">
-        <v>65.56999999999999</v>
-      </c>
+      <c r="H45" s="3" t="n"/>
       <c r="I45" s="3" t="n"/>
       <c r="J45" s="3" t="n"/>
       <c r="K45" s="4">
@@ -2176,6 +2803,29 @@
         <f>IF(AND(K45&gt;=80, K45&lt;=100), "4", IF(AND(K45&gt;=70, K45&lt;=79.99999999999), "3", IF(AND(K45&gt;=60, K45&lt;=69.9999999999), "2", IF(AND(K45&gt;=51, K45&lt;=59.999999999), "1", IF(AND(K45&gt;=0, K45&lt;=50.999999999), "0",  "0"  )  )  )  )  ) </f>
         <v/>
       </c>
+      <c r="N45" t="inlineStr">
+        <is>
+          <t>|</t>
+        </is>
+      </c>
+      <c r="O45" t="n">
+        <v>9.67</v>
+      </c>
+      <c r="P45" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q45" t="n">
+        <v>10</v>
+      </c>
+      <c r="R45" t="n">
+        <v>6.5</v>
+      </c>
+      <c r="S45" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="T45" t="n">
+        <v>80</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="0" t="inlineStr">
@@ -2197,13 +2847,9 @@
         </is>
       </c>
       <c r="E46" s="3" t="n"/>
-      <c r="F46" s="3" t="n">
-        <v>84.33</v>
-      </c>
+      <c r="F46" s="3" t="n"/>
       <c r="G46" s="3" t="n"/>
-      <c r="H46" s="3" t="n">
-        <v>88.87</v>
-      </c>
+      <c r="H46" s="3" t="n"/>
       <c r="I46" s="3" t="n"/>
       <c r="J46" s="3" t="n"/>
       <c r="K46" s="4">
@@ -2218,6 +2864,29 @@
         <f>IF(AND(K46&gt;=80, K46&lt;=100), "4", IF(AND(K46&gt;=70, K46&lt;=79.99999999999), "3", IF(AND(K46&gt;=60, K46&lt;=69.9999999999), "2", IF(AND(K46&gt;=51, K46&lt;=59.999999999), "1", IF(AND(K46&gt;=0, K46&lt;=50.999999999), "0",  "0"  )  )  )  )  ) </f>
         <v/>
       </c>
+      <c r="N46" t="inlineStr">
+        <is>
+          <t>|</t>
+        </is>
+      </c>
+      <c r="O46" t="n">
+        <v>8.33</v>
+      </c>
+      <c r="P46" t="n">
+        <v>10</v>
+      </c>
+      <c r="Q46" t="n">
+        <v>8.33</v>
+      </c>
+      <c r="R46" t="n">
+        <v>7.5</v>
+      </c>
+      <c r="S46" t="n">
+        <v>8.800000000000001</v>
+      </c>
+      <c r="T46" t="n">
+        <v>90</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="0" t="inlineStr">
@@ -2239,13 +2908,9 @@
         </is>
       </c>
       <c r="E47" s="3" t="n"/>
-      <c r="F47" s="3" t="n">
-        <v>28.67</v>
-      </c>
+      <c r="F47" s="3" t="n"/>
       <c r="G47" s="3" t="n"/>
-      <c r="H47" s="3" t="n">
-        <v>0</v>
-      </c>
+      <c r="H47" s="3" t="n"/>
       <c r="I47" s="3" t="n"/>
       <c r="J47" s="4" t="n"/>
       <c r="K47" s="4">
@@ -2260,6 +2925,20 @@
         <f>IF(AND(K47&gt;=80, K47&lt;=100), "4", IF(AND(K47&gt;=70, K47&lt;=79.99999999999), "3", IF(AND(K47&gt;=60, K47&lt;=69.9999999999), "2", IF(AND(K47&gt;=51, K47&lt;=59.999999999), "1", IF(AND(K47&gt;=0, K47&lt;=50.999999999), "0",  "0"  )  )  )  )  ) </f>
         <v/>
       </c>
+      <c r="N47" t="inlineStr">
+        <is>
+          <t>|</t>
+        </is>
+      </c>
+      <c r="Q47" t="n">
+        <v>0</v>
+      </c>
+      <c r="S47" t="n">
+        <v>8.6</v>
+      </c>
+      <c r="T47" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="0" t="inlineStr">
@@ -2281,13 +2960,9 @@
         </is>
       </c>
       <c r="E48" s="3" t="n"/>
-      <c r="F48" s="3" t="n">
-        <v>83.33</v>
-      </c>
+      <c r="F48" s="3" t="n"/>
       <c r="G48" s="3" t="n"/>
-      <c r="H48" s="3" t="n">
-        <v>46.67</v>
-      </c>
+      <c r="H48" s="3" t="n"/>
       <c r="I48" s="3" t="n"/>
       <c r="J48" s="3" t="n"/>
       <c r="K48" s="4">
@@ -2302,6 +2977,29 @@
         <f>IF(AND(K48&gt;=80, K48&lt;=100), "4", IF(AND(K48&gt;=70, K48&lt;=79.99999999999), "3", IF(AND(K48&gt;=60, K48&lt;=69.9999999999), "2", IF(AND(K48&gt;=51, K48&lt;=59.999999999), "1", IF(AND(K48&gt;=0, K48&lt;=50.999999999), "0",  "0"  )  )  )  )  ) </f>
         <v/>
       </c>
+      <c r="N48" t="inlineStr">
+        <is>
+          <t>|</t>
+        </is>
+      </c>
+      <c r="O48" t="n">
+        <v>9</v>
+      </c>
+      <c r="P48" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q48" t="n">
+        <v>5</v>
+      </c>
+      <c r="R48" t="n">
+        <v>7</v>
+      </c>
+      <c r="S48" t="n">
+        <v>9</v>
+      </c>
+      <c r="T48" t="n">
+        <v>90</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="0" t="inlineStr">
@@ -2323,13 +3021,9 @@
         </is>
       </c>
       <c r="E49" s="3" t="n"/>
-      <c r="F49" s="3" t="n">
-        <v>59.33</v>
-      </c>
+      <c r="F49" s="3" t="n"/>
       <c r="G49" s="3" t="n"/>
-      <c r="H49" s="3" t="n">
-        <v>98.90000000000001</v>
-      </c>
+      <c r="H49" s="3" t="n"/>
       <c r="I49" s="3" t="n"/>
       <c r="J49" s="3" t="n"/>
       <c r="K49" s="4">
@@ -2344,6 +3038,29 @@
         <f>IF(AND(K49&gt;=80, K49&lt;=100), "4", IF(AND(K49&gt;=70, K49&lt;=79.99999999999), "3", IF(AND(K49&gt;=60, K49&lt;=69.9999999999), "2", IF(AND(K49&gt;=51, K49&lt;=59.999999999), "1", IF(AND(K49&gt;=0, K49&lt;=50.999999999), "0",  "0"  )  )  )  )  ) </f>
         <v/>
       </c>
+      <c r="N49" t="inlineStr">
+        <is>
+          <t>|</t>
+        </is>
+      </c>
+      <c r="O49" t="n">
+        <v>9.67</v>
+      </c>
+      <c r="P49" t="n">
+        <v>10</v>
+      </c>
+      <c r="Q49" t="n">
+        <v>10</v>
+      </c>
+      <c r="R49" t="n">
+        <v>8.5</v>
+      </c>
+      <c r="S49" t="n">
+        <v>9.300000000000001</v>
+      </c>
+      <c r="T49" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="0" t="inlineStr">
@@ -2365,13 +3082,9 @@
         </is>
       </c>
       <c r="E50" s="3" t="n"/>
-      <c r="F50" s="3" t="n">
-        <v>86</v>
-      </c>
+      <c r="F50" s="3" t="n"/>
       <c r="G50" s="3" t="n"/>
-      <c r="H50" s="3" t="n">
-        <v>67.2</v>
-      </c>
+      <c r="H50" s="3" t="n"/>
       <c r="I50" s="3" t="n"/>
       <c r="J50" s="3" t="n"/>
       <c r="K50" s="4">
@@ -2386,6 +3099,29 @@
         <f>IF(AND(K50&gt;=80, K50&lt;=100), "4", IF(AND(K50&gt;=70, K50&lt;=79.99999999999), "3", IF(AND(K50&gt;=60, K50&lt;=69.9999999999), "2", IF(AND(K50&gt;=51, K50&lt;=59.999999999), "1", IF(AND(K50&gt;=0, K50&lt;=50.999999999), "0",  "0"  )  )  )  )  ) </f>
         <v/>
       </c>
+      <c r="N50" t="inlineStr">
+        <is>
+          <t>|</t>
+        </is>
+      </c>
+      <c r="O50" t="n">
+        <v>9.33</v>
+      </c>
+      <c r="P50" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="Q50" t="n">
+        <v>8.33</v>
+      </c>
+      <c r="R50" t="n">
+        <v>7.8</v>
+      </c>
+      <c r="S50" t="n">
+        <v>9</v>
+      </c>
+      <c r="T50" t="n">
+        <v>90</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="0" t="inlineStr">
@@ -2407,13 +3143,9 @@
         </is>
       </c>
       <c r="E51" s="3" t="n"/>
-      <c r="F51" s="3" t="n">
-        <v>55.67</v>
-      </c>
+      <c r="F51" s="3" t="n"/>
       <c r="G51" s="3" t="n"/>
-      <c r="H51" s="3" t="n">
-        <v>75.53</v>
-      </c>
+      <c r="H51" s="3" t="n"/>
       <c r="I51" s="3" t="n"/>
       <c r="J51" s="3" t="n"/>
       <c r="K51" s="4">
@@ -2428,6 +3160,29 @@
         <f>IF(AND(K51&gt;=80, K51&lt;=100), "4", IF(AND(K51&gt;=70, K51&lt;=79.99999999999), "3", IF(AND(K51&gt;=60, K51&lt;=69.9999999999), "2", IF(AND(K51&gt;=51, K51&lt;=59.999999999), "1", IF(AND(K51&gt;=0, K51&lt;=50.999999999), "0",  "0"  )  )  )  )  ) </f>
         <v/>
       </c>
+      <c r="N51" t="inlineStr">
+        <is>
+          <t>|</t>
+        </is>
+      </c>
+      <c r="O51" t="n">
+        <v>9.33</v>
+      </c>
+      <c r="P51" t="n">
+        <v>5</v>
+      </c>
+      <c r="Q51" t="n">
+        <v>8.33</v>
+      </c>
+      <c r="R51" t="n">
+        <v>8</v>
+      </c>
+      <c r="S51" t="n">
+        <v>8.699999999999999</v>
+      </c>
+      <c r="T51" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="0" t="inlineStr">
@@ -2449,13 +3204,9 @@
         </is>
       </c>
       <c r="E52" s="3" t="n"/>
-      <c r="F52" s="3" t="n">
-        <v>31.67</v>
-      </c>
+      <c r="F52" s="3" t="n"/>
       <c r="G52" s="3" t="n"/>
-      <c r="H52" s="3" t="n">
-        <v>73.90000000000001</v>
-      </c>
+      <c r="H52" s="3" t="n"/>
       <c r="I52" s="3" t="n"/>
       <c r="J52" s="3" t="n"/>
       <c r="K52" s="4">
@@ -2470,6 +3221,26 @@
         <f>IF(AND(K52&gt;=80, K52&lt;=100), "4", IF(AND(K52&gt;=70, K52&lt;=79.99999999999), "3", IF(AND(K52&gt;=60, K52&lt;=69.9999999999), "2", IF(AND(K52&gt;=51, K52&lt;=59.999999999), "1", IF(AND(K52&gt;=0, K52&lt;=50.999999999), "0",  "0"  )  )  )  )  ) </f>
         <v/>
       </c>
+      <c r="N52" t="inlineStr">
+        <is>
+          <t>|</t>
+        </is>
+      </c>
+      <c r="O52" t="n">
+        <v>8</v>
+      </c>
+      <c r="P52" t="n">
+        <v>7.5</v>
+      </c>
+      <c r="Q52" t="n">
+        <v>6.67</v>
+      </c>
+      <c r="S52" t="n">
+        <v>9.5</v>
+      </c>
+      <c r="T52" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="0" t="inlineStr">
@@ -2491,13 +3262,9 @@
         </is>
       </c>
       <c r="E53" s="3" t="n"/>
-      <c r="F53" s="3" t="n">
-        <v>21.67</v>
-      </c>
+      <c r="F53" s="3" t="n"/>
       <c r="G53" s="3" t="n"/>
-      <c r="H53" s="3" t="n">
-        <v>65.53</v>
-      </c>
+      <c r="H53" s="3" t="n"/>
       <c r="I53" s="3" t="n"/>
       <c r="J53" s="3" t="n"/>
       <c r="K53" s="4">
@@ -2512,6 +3279,26 @@
         <f>IF(AND(K53&gt;=80, K53&lt;=100), "4", IF(AND(K53&gt;=70, K53&lt;=79.99999999999), "3", IF(AND(K53&gt;=60, K53&lt;=69.9999999999), "2", IF(AND(K53&gt;=51, K53&lt;=59.999999999), "1", IF(AND(K53&gt;=0, K53&lt;=50.999999999), "0",  "0"  )  )  )  )  ) </f>
         <v/>
       </c>
+      <c r="N53" t="inlineStr">
+        <is>
+          <t>|</t>
+        </is>
+      </c>
+      <c r="O53" t="n">
+        <v>6.33</v>
+      </c>
+      <c r="P53" t="n">
+        <v>5</v>
+      </c>
+      <c r="Q53" t="n">
+        <v>8.33</v>
+      </c>
+      <c r="R53" t="n">
+        <v>7.5</v>
+      </c>
+      <c r="T53" t="n">
+        <v>-10</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="0" t="inlineStr">
@@ -2533,13 +3320,9 @@
         </is>
       </c>
       <c r="E54" s="3" t="n"/>
-      <c r="F54" s="3" t="n">
-        <v>84.67</v>
-      </c>
+      <c r="F54" s="3" t="n"/>
       <c r="G54" s="3" t="n"/>
-      <c r="H54" s="3" t="n">
-        <v>76.67</v>
-      </c>
+      <c r="H54" s="3" t="n"/>
       <c r="I54" s="3" t="n"/>
       <c r="J54" s="3" t="n"/>
       <c r="K54" s="4">
@@ -2554,6 +3337,29 @@
         <f>IF(AND(K54&gt;=80, K54&lt;=100), "4", IF(AND(K54&gt;=70, K54&lt;=79.99999999999), "3", IF(AND(K54&gt;=60, K54&lt;=69.9999999999), "2", IF(AND(K54&gt;=51, K54&lt;=59.999999999), "1", IF(AND(K54&gt;=0, K54&lt;=50.999999999), "0",  "0"  )  )  )  )  ) </f>
         <v/>
       </c>
+      <c r="N54" t="inlineStr">
+        <is>
+          <t>|</t>
+        </is>
+      </c>
+      <c r="O54" t="n">
+        <v>8</v>
+      </c>
+      <c r="P54" t="n">
+        <v>10</v>
+      </c>
+      <c r="Q54" t="n">
+        <v>5</v>
+      </c>
+      <c r="R54" t="n">
+        <v>8.199999999999999</v>
+      </c>
+      <c r="S54" t="n">
+        <v>9</v>
+      </c>
+      <c r="T54" t="n">
+        <v>82</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="0" t="inlineStr">
@@ -2575,13 +3381,9 @@
         </is>
       </c>
       <c r="E55" s="3" t="n"/>
-      <c r="F55" s="3" t="n">
-        <v>41.67</v>
-      </c>
+      <c r="F55" s="3" t="n"/>
       <c r="G55" s="3" t="n"/>
-      <c r="H55" s="3" t="n">
-        <v>0</v>
-      </c>
+      <c r="H55" s="3" t="n"/>
       <c r="I55" s="3" t="n"/>
       <c r="J55" s="3" t="n"/>
       <c r="K55" s="4">
@@ -2595,6 +3397,23 @@
       <c r="M55" s="0">
         <f>IF(AND(K55&gt;=80, K55&lt;=100), "4", IF(AND(K55&gt;=70, K55&lt;=79.99999999999), "3", IF(AND(K55&gt;=60, K55&lt;=69.9999999999), "2", IF(AND(K55&gt;=51, K55&lt;=59.999999999), "1", IF(AND(K55&gt;=0, K55&lt;=50.999999999), "0",  "0"  )  )  )  )  ) </f>
         <v/>
+      </c>
+      <c r="N55" t="inlineStr">
+        <is>
+          <t>|</t>
+        </is>
+      </c>
+      <c r="P55" t="n">
+        <v>0</v>
+      </c>
+      <c r="R55" t="n">
+        <v>4</v>
+      </c>
+      <c r="S55" t="n">
+        <v>8.5</v>
+      </c>
+      <c r="T55" t="n">
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>